<commit_message>
Ajustes de nombres del menu y comentarios del codigo
</commit_message>
<xml_diff>
--- a/reporte_logistica_barcos.xlsx
+++ b/reporte_logistica_barcos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen Ejecutivo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Inventario Paquetes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Optimización Mochila" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Rutas Óptimas Dijkstra" sheetId="4" state="visible" r:id="rId4"/>
@@ -522,7 +522,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="98" customWidth="1" min="2" max="2"/>
+    <col width="68" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
@@ -531,17 +531,17 @@
   </cols>
   <sheetData>
     <row r="1"/>
-    <row r="2" ht="35" customHeight="1">
+    <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>SISTEMA MULTIMODAL DE TRANSPORTE Y LOGÍSTICA</t>
+          <t>REPORTE DE ENTREGAS Y RUTAS</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Optimización de Cargas (Mochila 0/1) y Enrutamiento Óptimo (Dijkstra) | Uniminuto 6to Semestre</t>
+          <t>Resumen de optimizacion de paquetes (Mochila) y rutas (Dijkstra)</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1313,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Buque Portacontenedores Tolima</t>
+          <t>Barco Portacontenedores</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Boeing 777F Cargo Express</t>
+          <t>Avion de Carga</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Furgón Distribución Ibagué (Chevrolet FTR)</t>
+          <t>Furgon</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Van Urbana Ibagué (Renault Master)</t>
+          <t>Van</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Moto Reparto Ibagué (Yamaha Cargo)</t>
+          <t>Moto</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Enfocar proyecto exclusivamente en Barcos y rutas entre puertos
</commit_message>
<xml_diff>
--- a/reporte_logistica_barcos.xlsx
+++ b/reporte_logistica_barcos.xlsx
@@ -581,32 +581,32 @@
     <row r="6" ht="36" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>20,829.5 kg</t>
+          <t>38,550.0 kg</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>59.20 m³</t>
+          <t>80.31 m³</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>26.5%</t>
+          <t>20.1%</t>
         </is>
       </c>
     </row>
@@ -625,18 +625,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
@@ -716,7 +716,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Maquinaria Textil Industrial (Contenedor)</t>
+          <t>Contenedor de Maquinaria Textil</t>
         </is>
       </c>
       <c r="C2" s="6" t="n">
@@ -741,14 +741,14 @@
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>Ibagué - Picaleña / Parque Ind. (Comuna 9)</t>
+          <t>Puerto de Buenaventura (Colombia)</t>
         </is>
       </c>
       <c r="J2" s="6" t="n">
-        <v>4.4082</v>
+        <v>3.8833</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>-75.1583</v>
+        <v>-77.0333</v>
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Lote Repuestos Automotrices Pesados</t>
+          <t>Lote Repuestos Automotrices</t>
         </is>
       </c>
       <c r="C3" s="9" t="n">
@@ -790,14 +790,14 @@
       </c>
       <c r="I3" s="10" t="inlineStr">
         <is>
-          <t>Ibagué - Mirolindo (Comuna 9)</t>
+          <t>Puerto de Cartagena (Colombia)</t>
         </is>
       </c>
       <c r="J3" s="9" t="n">
-        <v>4.4251</v>
+        <v>10.391</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>-75.19889999999999</v>
+        <v>-75.4794</v>
       </c>
       <c r="L3" s="11" t="inlineStr">
         <is>
@@ -839,14 +839,14 @@
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Ibagué - Picaleña / Parque Ind. (Comuna 9)</t>
+          <t>Puerto de Buenaventura (Colombia)</t>
         </is>
       </c>
       <c r="J4" s="6" t="n">
-        <v>4.4082</v>
+        <v>3.8833</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>-75.1583</v>
+        <v>-77.0333</v>
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
@@ -863,47 +863,47 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Equipos Médicos de Alta Precisión (Urgente)</t>
+          <t>Cargamento Motores Industriales</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>1.1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>1.188</v>
+        <v>4.48</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>180</v>
+        <v>4200</v>
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>Aeropuerto Miami Internacional (MIA)</t>
+          <t>Puerto de Los Ángeles (EE.UU.)</t>
         </is>
       </c>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>Ibagué - Zona Centro (Comuna 1)</t>
+          <t>Puerto de Buenaventura (Colombia)</t>
         </is>
       </c>
       <c r="J5" s="9" t="n">
-        <v>4.4446</v>
+        <v>3.8833</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>-75.241</v>
+        <v>-77.0333</v>
       </c>
       <c r="L5" s="11" t="inlineStr">
         <is>
-          <t>AVION</t>
+          <t>BARCO</t>
         </is>
       </c>
       <c r="M5" s="9" t="n">
-        <v>98</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -912,47 +912,47 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Servidores y Racks de Telecomunicaciones</t>
+          <t>Equipos Eléctricos de Distribución</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>1.6</v>
+        <v>4.32</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>420</v>
+        <v>3800</v>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Aeropuerto Shanghái Pudong (PVG)</t>
+          <t>Puerto de Rotterdam (Países Bajos)</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Ibagué - Mirolindo (Comuna 9)</t>
+          <t>Puerto de Barranquilla (Colombia)</t>
         </is>
       </c>
       <c r="J6" s="6" t="n">
-        <v>4.4251</v>
+        <v>10.9685</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>-75.19889999999999</v>
+        <v>-74.7813</v>
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>AVION</t>
+          <t>BARCO</t>
         </is>
       </c>
       <c r="M6" s="6" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -961,7 +961,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Insumos Químicos y Fertilizantes Agrícolas</t>
+          <t>Insumos Químicos en Tambores</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
@@ -986,14 +986,14 @@
       </c>
       <c r="I7" s="10" t="inlineStr">
         <is>
-          <t>Ibagué - El Salado (Comuna 7)</t>
+          <t>Puerto de Cartagena (Colombia)</t>
         </is>
       </c>
       <c r="J7" s="9" t="n">
-        <v>4.4764</v>
+        <v>10.391</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>-75.18559999999999</v>
+        <v>-75.4794</v>
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Electrodomésticos y Neveras Comerciales</t>
+          <t>Electrodomésticos y Línea Blanca</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
@@ -1026,7 +1026,7 @@
         <v>2.508</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>850</v>
+        <v>2850</v>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
@@ -1035,14 +1035,14 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Ibagué - Mirolindo (Comuna 9)</t>
+          <t>Puerto de Santa Marta (Colombia)</t>
         </is>
       </c>
       <c r="J8" s="6" t="n">
-        <v>4.4251</v>
+        <v>11.2408</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>-75.19889999999999</v>
+        <v>-74.199</v>
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
@@ -1059,23 +1059,23 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Cajas de Calzado y Textiles para Comercio</t>
+          <t>Cajas de Calzado y Textiles</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>0.432</v>
+        <v>1.8</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>95</v>
+        <v>1500</v>
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
@@ -1084,14 +1084,14 @@
       </c>
       <c r="I9" s="10" t="inlineStr">
         <is>
-          <t>Ibagué - Zona Centro (Comuna 1)</t>
+          <t>Puerto de Barranquilla (Colombia)</t>
         </is>
       </c>
       <c r="J9" s="9" t="n">
-        <v>4.4446</v>
+        <v>10.9685</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>-75.241</v>
+        <v>-74.7813</v>
       </c>
       <c r="L9" s="11" t="inlineStr">
         <is>
@@ -1108,47 +1108,47 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Medicamentos Refrigerados y Vacunas</t>
+          <t>Contenedor de Paneles Solares</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.6</v>
+        <v>2.2</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.15</v>
+        <v>11.55</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>28</v>
+        <v>4600</v>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Aeropuerto Ámsterdam Schiphol (AMS)</t>
+          <t>Puerto de Rotterdam (Países Bajos)</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Ibagué - Zona Centro (Comuna 1)</t>
+          <t>Puerto de Santa Marta (Colombia)</t>
         </is>
       </c>
       <c r="J10" s="6" t="n">
-        <v>4.4446</v>
+        <v>11.2408</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>-75.241</v>
+        <v>-74.199</v>
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>AVION</t>
+          <t>BARCO</t>
         </is>
       </c>
       <c r="M10" s="6" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -1157,145 +1157,47 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Documentación Notarial y Contratos Urgentes</t>
+          <t>Herramientas y Ferretería Pesada</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>0.1</v>
+        <v>1.3</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>0.25</v>
+        <v>1.2</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>0.35</v>
+        <v>1.6</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>0.008999999999999999</v>
+        <v>2.496</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>3.5</v>
+        <v>2400</v>
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>Aeropuerto Bogotá El Dorado (BOG)</t>
+          <t>Puerto de Los Ángeles (EE.UU.)</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
         <is>
-          <t>Ibagué - Ricaurte (Comuna 12)</t>
+          <t>Puerto de Buenaventura (Colombia)</t>
         </is>
       </c>
       <c r="J11" s="9" t="n">
-        <v>4.4211</v>
+        <v>3.8833</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>-75.2415</v>
+        <v>-77.0333</v>
       </c>
       <c r="L11" s="11" t="inlineStr">
         <is>
-          <t>AVION</t>
+          <t>BARCO</t>
         </is>
       </c>
       <c r="M11" s="9" t="n">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="6" t="n">
-        <v>111</v>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Paquete Repuestos de Drones y Microelectrónica</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>Aeropuerto Shanghái Pudong (PVG)</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="inlineStr">
-        <is>
-          <t>Ibagué - Zona Centro (Comuna 1)</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="n">
-        <v>4.4446</v>
-      </c>
-      <c r="K12" s="6" t="n">
-        <v>-75.241</v>
-      </c>
-      <c r="L12" s="8" t="inlineStr">
-        <is>
-          <t>AVION</t>
-        </is>
-      </c>
-      <c r="M12" s="6" t="n">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="9" t="n">
-        <v>112</v>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Caja Herramientas Eléctricas para Taller</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F13" s="9" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>45</v>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>Puerto de Rotterdam (Países Bajos)</t>
-        </is>
-      </c>
-      <c r="I13" s="10" t="inlineStr">
-        <is>
-          <t>Ibagué - El Salado (Comuna 7)</t>
-        </is>
-      </c>
-      <c r="J13" s="9" t="n">
-        <v>4.4764</v>
-      </c>
-      <c r="K13" s="9" t="n">
-        <v>-75.18559999999999</v>
-      </c>
-      <c r="L13" s="11" t="inlineStr">
-        <is>
-          <t>BARCO</t>
-        </is>
-      </c>
-      <c r="M13" s="9" t="n">
-        <v>50</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1309,12 +1211,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -1322,23 +1224,23 @@
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="37" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>ID Vehículo</t>
+          <t>ID Barco</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>Nombre de Transporte</t>
+          <t>Nombre del Barco</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>Tipo Modal</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
@@ -1399,221 +1301,33 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>60000</v>
+        <v>25000</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>20190</v>
+        <v>24650</v>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>33.65%</t>
+          <t>98.6%</t>
         </is>
       </c>
       <c r="G2" s="6" t="n">
-        <v>450</v>
+        <v>180</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>56.214</v>
+        <v>36.118</v>
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>12.49%</t>
+          <t>20.07%</t>
         </is>
       </c>
       <c r="J2" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>101, 102, 103, 106, 107, 108, 112</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>AV-01</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>Avion de Carga</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="inlineStr">
-        <is>
-          <t>AVION</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="n">
-        <v>18000</v>
-      </c>
-      <c r="E3" s="9" t="n">
-        <v>639.5</v>
-      </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>3.55%</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="n">
-        <v>110</v>
-      </c>
-      <c r="H3" s="9" t="n">
-        <v>2.983</v>
-      </c>
-      <c r="I3" s="9" t="inlineStr">
-        <is>
-          <t>2.71%</t>
-        </is>
-      </c>
-      <c r="J3" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>104, 105, 109, 110, 111</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>FUR-01</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Furgon</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>FURGON</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>4000</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>3200</v>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>80.0%</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>5.94</v>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>27.0%</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="7" t="inlineStr">
-        <is>
-          <t>102</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>VAN-01</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Van</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>VAN</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E5" s="9" t="n">
-        <v>740</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>61.67%</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="H5" s="9" t="n">
-        <v>3.34</v>
-      </c>
-      <c r="I5" s="9" t="inlineStr">
-        <is>
-          <t>37.11%</t>
-        </is>
-      </c>
-      <c r="J5" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="K5" s="10" t="inlineStr">
-        <is>
-          <t>104, 105, 108, 112</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>MOT-01</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Moto</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>MOTO</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>90.0%</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>0.159</v>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>53.0%</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K6" s="7" t="inlineStr">
-        <is>
-          <t>109, 110</t>
+          <t>102, 104, 105, 106, 107, 108, 109, 110</t>
         </is>
       </c>
     </row>
@@ -1628,16 +1342,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="169" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="4" max="4"/>
+    <col width="170" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="27" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1654,17 +1368,17 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>Nodo Origen</t>
+          <t>Puerto Origen</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>Destino en Ibagué</t>
+          <t>Puerto Destino</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>Ruta Óptima Calculada</t>
+          <t>Ruta Marítima Óptima</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
@@ -1674,7 +1388,7 @@
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>Distancia Total (km)</t>
+          <t>Distancia Náutica (km)</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
@@ -1689,7 +1403,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Maquinaria Textil Industrial (Contenedor)</t>
+          <t>Contenedor de Maquinaria Textil</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
@@ -1699,22 +1413,22 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>Ibagué - Picaleña / Parque Ind. (Comuna 9)</t>
+          <t>Puerto de Buenaventura (Colombia)</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>Puerto de Shanghái (China) ➔ Puerto de Buenaventura (Col - Pacífico) ➔ Cali (Hub Pacífico) ➔ Ibagué (Hub Central Tolima) ➔ Ibagué - Picaleña / Parque Ind. (Comuna 9)</t>
+          <t>Puerto de Shanghái (China) ➔ Puerto de Buenaventura (Colombia)</t>
         </is>
       </c>
       <c r="F2" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>15776.8</v>
+        <v>15400</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>393.85</v>
+        <v>385</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -1723,7 +1437,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Lote Repuestos Automotrices Pesados</t>
+          <t>Lote Repuestos Automotrices</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
@@ -1733,22 +1447,22 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>Ibagué - Mirolindo (Comuna 9)</t>
+          <t>Puerto de Cartagena (Colombia)</t>
         </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
-          <t>Puerto de Rotterdam (Países Bajos) ➔ Puerto de Cartagena (Col - Caribe) ➔ Medellín (Hub Central) ➔ Ibagué (Hub Central Tolima) ➔ Ibagué - Mirolindo (Comuna 9)</t>
+          <t>Puerto de Rotterdam (Países Bajos) ➔ Puerto de Cartagena (Colombia)</t>
         </is>
       </c>
       <c r="F3" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>9436.200000000001</v>
+        <v>8400</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>229.6</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -1767,22 +1481,22 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Ibagué - Picaleña / Parque Ind. (Comuna 9)</t>
+          <t>Puerto de Buenaventura (Colombia)</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Puerto de Shanghái (China) ➔ Puerto de Buenaventura (Col - Pacífico) ➔ Cali (Hub Pacífico) ➔ Ibagué (Hub Central Tolima) ➔ Ibagué - Picaleña / Parque Ind. (Comuna 9)</t>
+          <t>Puerto de Shanghái (China) ➔ Puerto de Buenaventura (Colombia)</t>
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>15776.8</v>
+        <v>15400</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>393.85</v>
+        <v>385</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -1791,32 +1505,32 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Equipos Médicos de Alta Precisión (Urgente)</t>
+          <t>Cargamento Motores Industriales</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Aeropuerto Miami Internacional (MIA)</t>
+          <t>Puerto de Los Ángeles (EE.UU.)</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Ibagué - Zona Centro (Comuna 1)</t>
+          <t>Puerto de Buenaventura (Colombia)</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>Aeropuerto Miami Internacional (MIA) ➔ Aeropuerto Bogotá El Dorado (BOG) ➔ Ibagué (Hub Central Tolima) ➔ Ibagué - Zona Centro (Comuna 1)</t>
+          <t>Puerto de Los Ángeles (EE.UU.) ➔ Puerto de Buenaventura (Colombia)</t>
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>2634.5</v>
+        <v>5500</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>8.25</v>
+        <v>137.5</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -1825,32 +1539,32 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Servidores y Racks de Telecomunicaciones</t>
+          <t>Equipos Eléctricos de Distribución</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Aeropuerto Shanghái Pudong (PVG)</t>
+          <t>Puerto de Rotterdam (Países Bajos)</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Ibagué - Mirolindo (Comuna 9)</t>
+          <t>Puerto de Barranquilla (Colombia)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Aeropuerto Shanghái Pudong (PVG) ➔ Aeropuerto Bogotá El Dorado (BOG) ➔ Ibagué (Hub Central Tolima) ➔ Ibagué - Mirolindo (Comuna 9)</t>
+          <t>Puerto de Rotterdam (Países Bajos) ➔ Puerto de Cartagena (Colombia) ➔ Puerto de Barranquilla (Colombia)</t>
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>16006.2</v>
+        <v>8520</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>24</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -1859,7 +1573,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Insumos Químicos y Fertilizantes Agrícolas</t>
+          <t>Insumos Químicos en Tambores</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -1869,22 +1583,22 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Ibagué - El Salado (Comuna 7)</t>
+          <t>Puerto de Cartagena (Colombia)</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>Puerto de Miami (EE.UU.) ➔ Puerto de Cartagena (Col - Caribe) ➔ Medellín (Hub Central) ➔ Ibagué (Hub Central Tolima) ➔ Ibagué - El Salado (Comuna 7)</t>
+          <t>Puerto de Miami (EE.UU.) ➔ Puerto de Cartagena (Colombia)</t>
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>2841.2</v>
+        <v>1800</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>64.75</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -1893,7 +1607,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Electrodomésticos y Neveras Comerciales</t>
+          <t>Electrodomésticos y Línea Blanca</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -1903,22 +1617,22 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Ibagué - Mirolindo (Comuna 9)</t>
+          <t>Puerto de Santa Marta (Colombia)</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Puerto de Shanghái (China) ➔ Puerto de Buenaventura (Col - Pacífico) ➔ Cali (Hub Pacífico) ➔ Ibagué (Hub Central Tolima) ➔ Ibagué - Mirolindo (Comuna 9)</t>
+          <t>Puerto de Shanghái (China) ➔ Puerto de Buenaventura (Colombia) ➔ Puerto de Cartagena (Colombia) ➔ Puerto de Barranquilla (Colombia) ➔ Puerto de Santa Marta (Colombia)</t>
         </is>
       </c>
       <c r="F8" s="6" t="n">
         <v>4</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>15773.2</v>
+        <v>16355</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>393.8</v>
+        <v>408.6</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -1927,7 +1641,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Cajas de Calzado y Textiles para Comercio</t>
+          <t>Cajas de Calzado y Textiles</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
@@ -1937,22 +1651,22 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Ibagué - Zona Centro (Comuna 1)</t>
+          <t>Puerto de Barranquilla (Colombia)</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Puerto de Miami (EE.UU.) ➔ Puerto de Cartagena (Col - Caribe) ➔ Medellín (Hub Central) ➔ Ibagué (Hub Central Tolima) ➔ Ibagué - Zona Centro (Comuna 1)</t>
+          <t>Puerto de Miami (EE.UU.) ➔ Puerto de Cartagena (Colombia) ➔ Puerto de Barranquilla (Colombia)</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>2834.5</v>
+        <v>1920</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>64.55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -1961,32 +1675,32 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Medicamentos Refrigerados y Vacunas</t>
+          <t>Contenedor de Paneles Solares</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Aeropuerto Ámsterdam Schiphol (AMS)</t>
+          <t>Puerto de Rotterdam (Países Bajos)</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Ibagué - Zona Centro (Comuna 1)</t>
+          <t>Puerto de Santa Marta (Colombia)</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Aeropuerto Ámsterdam Schiphol (AMS) ➔ Aeropuerto Bogotá El Dorado (BOG) ➔ Ibagué (Hub Central Tolima) ➔ Ibagué - Zona Centro (Comuna 1)</t>
+          <t>Puerto de Rotterdam (Países Bajos) ➔ Puerto de Cartagena (Colombia) ➔ Puerto de Barranquilla (Colombia) ➔ Puerto de Santa Marta (Colombia)</t>
         </is>
       </c>
       <c r="F10" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>9054.5</v>
+        <v>8605</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>15.65</v>
+        <v>215.1</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -1995,100 +1709,32 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Documentación Notarial y Contratos Urgentes</t>
+          <t>Herramientas y Ferretería Pesada</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Aeropuerto Bogotá El Dorado (BOG)</t>
+          <t>Puerto de Los Ángeles (EE.UU.)</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Ibagué - Ricaurte (Comuna 12)</t>
+          <t>Puerto de Buenaventura (Colombia)</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>Aeropuerto Bogotá El Dorado (BOG) ➔ Ibagué (Hub Central Tolima) ➔ Ibagué - Ricaurte (Comuna 12)</t>
+          <t>Puerto de Los Ángeles (EE.UU.) ➔ Puerto de Buenaventura (Colombia)</t>
         </is>
       </c>
       <c r="F11" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>205.1</v>
+        <v>5500</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>4.48</v>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="6" t="n">
-        <v>111</v>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Paquete Repuestos de Drones y Microelectrónica</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Aeropuerto Shanghái Pudong (PVG)</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Ibagué - Zona Centro (Comuna 1)</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>Aeropuerto Shanghái Pudong (PVG) ➔ Aeropuerto Bogotá El Dorado (BOG) ➔ Ibagué (Hub Central Tolima) ➔ Ibagué - Zona Centro (Comuna 1)</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>16004.5</v>
-      </c>
-      <c r="H12" s="6" t="n">
-        <v>23.95</v>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="9" t="n">
-        <v>112</v>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Caja Herramientas Eléctricas para Taller</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>Puerto de Rotterdam (Países Bajos)</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>Ibagué - El Salado (Comuna 7)</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>Puerto de Rotterdam (Países Bajos) ➔ Puerto de Cartagena (Col - Caribe) ➔ Medellín (Hub Central) ➔ Ibagué (Hub Central Tolima) ➔ Ibagué - El Salado (Comuna 7)</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>9441.200000000001</v>
-      </c>
-      <c r="H13" s="9" t="n">
-        <v>229.75</v>
+        <v>137.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>